<commit_message>
Atualização planilha 14.09.2026 e remoção botão Custos Indiretos da página inicial
</commit_message>
<xml_diff>
--- a/Planilha de Despesas .xlsx
+++ b/Planilha de Despesas .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cliente/Downloads/Projeto Orçamento Gemini/Site DOR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cliente/Downloads/Projeto Orçamento Chatgpt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF2A8D50-9AF0-BD43-844E-5E57507D206E}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48317F3-8C17-5A40-A809-7E7EF38EE196}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15620" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="500" windowWidth="28800" windowHeight="15760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -6671,7 +6671,7 @@
       </c>
       <c r="F30" s="46" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>EXPIRADO</v>
+        <v>EM BREVE</v>
       </c>
       <c r="G30" s="29" t="s">
         <v>152</v>
@@ -6765,7 +6765,7 @@
       </c>
       <c r="F31" s="46" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>EM BREVE</v>
+        <v>NO PRAZO</v>
       </c>
       <c r="G31" s="46"/>
       <c r="H31" s="74" t="s">
@@ -12887,7 +12887,7 @@
       </c>
       <c r="G6" s="46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>EXPIRADO</v>
+        <v>EM BREVE</v>
       </c>
       <c r="H6" s="29" t="s">
         <v>152</v>
@@ -12949,7 +12949,7 @@
       </c>
       <c r="G7" s="46" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>EM BREVE</v>
+        <v>NO PRAZO</v>
       </c>
       <c r="H7" s="46"/>
       <c r="I7" s="74" t="s">
@@ -19179,7 +19179,7 @@
       </c>
       <c r="G30" s="46" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>EXPIRADO</v>
+        <v>EM BREVE</v>
       </c>
       <c r="H30" s="29" t="s">
         <v>152</v>
@@ -19279,7 +19279,7 @@
       </c>
       <c r="G31" s="46" t="str">
         <f t="shared" ca="1" si="4"/>
-        <v>EM BREVE</v>
+        <v>NO PRAZO</v>
       </c>
       <c r="H31" s="46"/>
       <c r="I31" s="74" t="s">

</xml_diff>